<commit_message>
stats and data added on the database, scraping was succesfull. Next step, completing adding serie a2 data
</commit_message>
<xml_diff>
--- a/scraper/SquadreBNazionale.xlsx
+++ b/scraper/SquadreBNazionale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\feder\OneDrive\Desktop\Tesi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5735950C-046A-4AD2-BD44-15DEFBAA0F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{209584D7-8075-4637-841E-38309D682F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -231,9 +231,6 @@
     <t>https://web.archive.org/web/20260619152955/https://www.legapallacanestro.com/serie-b/siaz-basket-piazza-armerina</t>
   </si>
   <si>
-    <t>https://web.archive.org/web/20260429164147/https://www.legapallacanestro.com/serie-b/rucker-san-vendemiano</t>
-  </si>
-  <si>
     <t>https://web.archive.org/web/20260622113109/https://www.legapallacanestro.com/serie-b/tav-treviglio-brianza-basket</t>
   </si>
   <si>
@@ -310,6 +307,9 @@
   </si>
   <si>
     <t>VIRTUS GVM ROMA 1960</t>
+  </si>
+  <si>
+    <t>https://web.archive.org/web/20260429115202/https://www.legapallacanestro.com/serie-b/rucker-san-vendemiano</t>
   </si>
 </sst>
 </file>
@@ -649,6 +649,7 @@
   <cols>
     <col min="1" max="1" width="40.44140625" customWidth="1"/>
     <col min="3" max="3" width="121.5546875" customWidth="1"/>
+    <col min="4" max="4" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -791,7 +792,7 @@
         <v>15</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -835,7 +836,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>54</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -846,7 +847,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -857,18 +858,18 @@
         <v>15</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B20" t="s">
         <v>15</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -879,7 +880,7 @@
         <v>31</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -890,7 +891,7 @@
         <v>31</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -901,7 +902,7 @@
         <v>31</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -912,7 +913,7 @@
         <v>31</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -923,7 +924,7 @@
         <v>31</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -934,7 +935,7 @@
         <v>31</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -945,7 +946,7 @@
         <v>31</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -956,7 +957,7 @@
         <v>31</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -967,7 +968,7 @@
         <v>31</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -978,7 +979,7 @@
         <v>31</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -989,7 +990,7 @@
         <v>31</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -1000,18 +1001,18 @@
         <v>31</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B33" t="s">
         <v>31</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -1022,7 +1023,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -1033,7 +1034,7 @@
         <v>31</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -1044,7 +1045,7 @@
         <v>31</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -1055,18 +1056,18 @@
         <v>31</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B38" t="s">
         <v>31</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -1077,7 +1078,7 @@
         <v>31</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>